<commit_message>
Reporting pipeline in English: outputs, source files, checks, summary, dashboard; readable PDFs
- every visible text is English: source file names and headers, workbook sheets and labels, check messages,
  board pack sentences (numbers as €1,234 and −8.9%), terminal output, report.md, dashboard pages
- verdicts: TIES / DOES NOT TIE; files: overview.xlsx, pivot.xlsx, summary.html, contract.json, CONTRACT.md
- one summary page (English); the Slovak variant is removed
- no figure changed: every numeric cell of overview.xlsx and pivot.xlsx equals the Slovak version to the cent;
  the same 13 checks fail on the delivery with planted errors; contract re-signed for the renamed delivery
- examples: board-pack.pdf and control-panel-with-errors.pdf rebuilt in landscape with wrapped text and a
  readable font; README pictures rebuilt from the same sheets
- code comments stay in Slovak

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/reporting-pipeline/board-pack.xlsx
+++ b/examples/reporting-pipeline/board-pack.xlsx
@@ -7,18 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prehľad" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="P&amp;L YTD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mesiace x strediská" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Plán vs skutočnosť" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Months x cost centres" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Plan vs actual" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Board pack" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Odhad roka" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Odchýlky" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Riziká a príležitosti" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Komentáre" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Kontroly" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Kontrolný panel" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Chybné riadky" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Full-year forecast" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Variances" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Risks and opportunities" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Comments" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Checks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Control panel" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Failed rows" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
   <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="73" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -453,38 +453,38 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>stav k 2026-09</t>
+          <t>as of 2026-09</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Verdikt</t>
+          <t>Verdict</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SEDÍ</t>
+          <t>TIES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zmluva reportu</t>
+          <t>Report contract</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ODOSLANIE POVOLENÉ — 17/17 čísel zmluvy z hotového prehlad.xlsx sedí s 2 kotvami mimo motora (±1 €; percentá = správne zaokrúhlená kotva) · zmluvu podpísal kontrolór (demo) 2026-09-27</t>
+          <t>RELEASE ALLOWED — 17/17 contract figures from the finished overview.xlsx tie to 2 anchors outside the engine (±€1; percentages = correctly rounded anchor) · contract signed by controller (demo) 2026-09-27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>YTD EBITDA (€)</t>
+          <t>EBITDA year to date (€)</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -494,7 +494,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>YTD tržby (€)</t>
+          <t>Revenue year to date (€)</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -505,7 +505,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Zistenia pre board</t>
+          <t>Findings for the board</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hračky: medziročný pokles 3 štvrťroky po sebe (Q1 −6,8 %, Q2 −13,5 %, Q3 −18,5 %)</t>
+          <t>Toys: year-on-year decline 3 quarters in a row (Q1 −6.8%, Q2 −13.5%, Q3 −18.5%)</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Odhad EBITDA roka (€)</t>
+          <t>Full-year EBITDA forecast (€)</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -535,7 +535,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Plán EBITDA roka (€)</t>
+          <t>Full-year EBITDA plan (€)</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
@@ -545,12 +545,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Metóda odhadu</t>
+          <t>Forecast method</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Odhad zvyšku roka: mesiac = plán mesiaca × (skutočnosť ÷ plán za posledné 3 mesiace) po stredisku a riadku; riadok bez plánu = priemer posledných 3 mesiacov; daň = 21 % × odhad zisku pred zdanením. Plán neobsahuje daň z príjmov — plán dane = 21 % × plán zisku pred zdanením mesiaca.</t>
+          <t>Rest-of-year forecast: month = month's plan × (actual ÷ plan for the last 3 months) by cost centre and line; a line without a plan = average of the last 3 months; tax = 21% × forecast profit before tax. The plan does not include income tax — plan tax = 21% × the month's planned profit before tax.</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Odhad roka</t>
+          <t>Full-year forecast</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tržby 2026 — odhad 2 122 954 €: voči plánu −8 532 € (−0,4 %), voči minulému roku +149 356 €; z toho skutočnosť 1 496 289 € a odhad zvyšku roka 626 665 €.</t>
+          <t>Revenue 2026 — forecast €2,122,954: vs plan −€8,532 (−0.4%), vs last year +€149,356; of which actual €1,496,289 and rest-of-year forecast €626,665.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EBITDA 2026 — odhad 241 296 €: voči plánu −23 660 € (−8,9 %), voči minulému roku +19 825 €; z toho skutočnosť 160 045 € a odhad zvyšku roka 81 251 €.</t>
+          <t>EBITDA 2026 — forecast €241,296: vs plan −€23,660 (−8.9%), vs last year +€19,825; of which actual €160,045 and rest-of-year forecast €81,251.</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Čistý zisk 2026 — odhad 149 246 €: voči plánu −17 233 € (−10,4 %), voči minulému roku +17 120 €; z toho skutočnosť 95 279 € a odhad zvyšku roka 53 967 €.</t>
+          <t>Net profit 2026 — forecast €149,246: vs plan −€17,233 (−10.4%), vs last year +€17,120; of which actual €95,279 and rest-of-year forecast €53,967.</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Najväčšie odchýlky voči plánu</t>
+          <t>Largest variances vs plan</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Predajňa OC · Nájom: vplyv na EBITDA −15 600 € voči plánu (−31,0 %) — od 2026-04 mesačne −2 600 €; voči minulému roku −15 600 €.</t>
+          <t>Store OC · Rent: EBITDA impact −€15,600 vs plan (−31.0%) — since 2026-04, every month −€2,600; vs last year −€15,600.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Predajňa Mesto · Hrubá marža: vplyv na EBITDA −3 904 € voči plánu (−4,4 %) — najmä v Q2 (−2 692 €); voči minulému roku +2 735 €.</t>
+          <t>Store Mesto · Gross margin: EBITDA impact −€3,904 vs plan (−4.4%) — mainly in Q2 (−€2,692); vs last year +€2,735.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Predajňa OC · Hrubá marža: vplyv na EBITDA +3 626 € voči plánu (+1,6 %) — najmä v Q3 (+5 421 €); voči minulému roku +20 919 €.</t>
+          <t>Store OC · Gross margin: EBITDA impact +€3,626 vs plan (+1.6%) — mainly in Q3 (+€5,421); vs last year +€20,919.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko · Hrubá marža: vplyv na EBITDA −3 286 € voči plánu (−2,7 %) — rozložené počas roka (priemer −365 € mesačne); voči minulému roku +5 738 €.</t>
+          <t>Store Sídlisko · Gross margin: EBITDA impact −€3,286 vs plan (−2.7%) — spread across the year (average −€365 per month); vs last year +€5,738.</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Riziká a príležitosti</t>
+          <t>Risks and opportunities</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Energie: v Q1 2026 +35,0 % medziročne, posledných 3 mesiacov +0,0 %; ak sa skok zopakuje vo zvyšku roka (minulý rok −5 083 € × 1,35), EBITDA −1 779 € voči odhadu.</t>
+          <t>Energy: in Q1 2026 +35.0% year on year, last 3 months +0.0%; if the spike repeats in the rest of the year (last year −€5,083 × 1.35), EBITDA −€1,779 vs forecast.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Citlivosť odhadu na metódu (položky sa prekrývajú — nesčítavať)</t>
+          <t>Forecast sensitivity to the method (items overlap — do not add them up)</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Papiernictvo (rast +21,9 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 52,9 % tržieb, vo zvyšku roka 33,8 %; oprava na podiel zvyšku roka: EBITDA −9 783 € (× hrubá marža).</t>
+          <t>Stationery (growth +21.9% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 52.9% share of revenue, in the rest of the year 33.8%; correction to the rest-of-year share: EBITDA −€9,783 (× gross margin).</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hračky (pokles −18,5 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 15,0 % tržieb, vo zvyšku roka 25,1 %; oprava na podiel zvyšku roka: EBITDA −4 356 € (× hrubá marža).</t>
+          <t>Toys (decline −18.5% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 15.0% share of revenue, in the rest of the year 25.1%; correction to the rest-of-year share: EBITDA −€4,356 (× gross margin).</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Čo som neoveroval</t>
+          <t>What was not checked</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>vecná správnosť zaúčtovania na účet — kontroly overujú párovanie zdrojov a súčty; stredisko a mesiac faktúr sa párujú s knihou faktúr</t>
+          <t>whether a posting is on the right account in substance — the checks verify the reconciliation of sources and totals; the cost centre and month of invoices are matched to the invoice register</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DPH — sadzby na bločkoch sa neoverujú voči kategórii; overuje sa tržba bez DPH (604) a súčet s DPH po dňoch a spôsobe platby</t>
+          <t>VAT — the rates on receipts are not checked against the category; what is checked is revenue excl. VAT (604) and the total incl. VAT by day and payment method</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>odpisy (551) — bez registra majetku sa neoverujú; daň z príjmov (591) je priebežný odhad 21 % zo zisku, neoverovaný voči priznaniu (overená je len úhrada preddavku 341 z banky — okrem posledného mesiaca obdobia, jeho úhrada príde až po období)</t>
+          <t>depreciation (551) — not checked without a fixed asset register; income tax (591) is an interim estimate of 21% of profit, not checked against the tax return (only the payment of the advance 341 from the bank is checked — except for the last month of the period, whose payment arrives after the period)</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>pravosť prvotných dokladov — falošný bloček zapísaný do pokladne aj SPOLU, alebo fiktívna faktúra dodávateľa z číselníka zaúčtovaná aj uhradená, prejde: párovanie zdroj ↔ zdroj z princípu nevidí zdroj sfalšovaný na začiatku</t>
+          <t>authenticity of source documents — a fake receipt entered in the POS and in TOTAL, or a fictitious invoice from a supplier in the master data that is posted and paid, will pass: source ↔ source reconciliation by design cannot see a source falsified at the start</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>kategória tovaru na bločku — jediný zdroj je pokladňa; presun tržieb medzi kategóriami s rovnakou sadzbou DPH sa neoverí</t>
+          <t>goods category on the receipt — the POS is the only source; a shift of revenue between categories with the same VAT rate is not detected</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>manko a odpis zásob — výdaj zo skladu bez predaja zapísaný konzistentne v sklade, denníku aj predvahe prejde</t>
+          <t>shortage and stock write-off — a stock issue without a sale recorded consistently in stock, journal and trial balance will pass</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>tolerancia 0,05 € na deň v párovaní tržieb bez DPH (zaokrúhlenie DPH na bločkoch) — za obdobie spolu najviac ~100 €</t>
+          <t>tolerance of €0.05 a day in the reconciliation of revenue excl. VAT (VAT rounding on receipts) — at most ~€100 for the whole period</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>stav bankového účtu voči skutočnej banke — overuje sa výpis sám so sebou a s účtovníctvom</t>
+          <t>bank account balance against the real bank — the statement is checked against itself and against the books</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>úhrady počiatočných záväzkov k 31.12.2024 sa párujú len so súvahou 321 (kniha faktúr začína v 2025)</t>
+          <t>payments of opening liabilities as at 2024-12-31 are matched only to balance sheet account 321 (the invoice register starts in 2025)</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>hodnoty plánu — len tvar (plán je zámer, nie fakt)</t>
+          <t>plan values — shape only (a plan is an intention, not a fact)</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>výnimky sú vypnuté do rozhodnutia vedenia — každý nález znamená NESEDÍ</t>
+          <t>exceptions are switched off until management decides — every finding means DOES NOT TIE</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1042 riadkov predvahy mimo výsledovky (triedy mimo 5/6, obraty 30,635,737.97 €) — do výsledovky nevstupujú a neoverovali sa</t>
+          <t>1042 trial balance rows outside the P&amp;L (classes other than 5/6, turnover €30,635,737.97) — they do not enter the P&amp;L and were not checked</t>
         </is>
       </c>
     </row>
@@ -880,12 +880,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Stav</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Kontrola</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>model 'retail_full', 21 kontrol profilu (povinné: 21/21)</t>
+          <t>model 'retail_full', 21 checks in the profile (required: 21/21)</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>dodávka = kontrakt (233 súborov)</t>
+          <t>delivery = contract (233 files)</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>382,560 riadkov z 10 tabuliek zdrojov prečítaných bez straty</t>
+          <t>382,560 rows from 10 source tables read without loss</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4,350 súm je číslo v dohodnutom tvare</t>
+          <t>4,350 amounts are numbers in the agreed format</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bločky, denník, faktúry, mzdy, banka aj predvaha bez duplicít</t>
+          <t>receipts, journal, invoices, payroll, bank and trial balance without duplicates</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21 mesiacov × 7 zdrojov a 4 pokladne × 21 mesiacov bez medzery</t>
+          <t>21 months × 7 sources and 4 POS × 21 months without a gap</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>84 exportov pokladne: SPOLU == súčet bločkov</t>
+          <t>84 POS exports: TOTAL == sum of receipts</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2,175 obratov mesiac × stredisko × účet: denník == predvaha na cent</t>
+          <t>2,175 turnovers month × cost centre × account: journal == trial balance to the cent</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2,088 predajných dní × predajňa: bločky == 211/315 po spôsobe platby a tržby bez DPH == celý účet 604</t>
+          <t>2,088 sales days × store: receipts == 211/315 by payment method and revenue excl. VAT == the whole account 604</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>21 výpisov: zostatky nadväzujú a sedia s pohybmi</t>
+          <t>21 statements: balances carry forward and tie to the movements</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>439 bankových dní: výpis == účet 221 na cent</t>
+          <t>439 bank days: statement == account 221 to the cent</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1,664 úhrad faktúr (VS, IČO, suma) a 4,784 menovitých interných platieb — žiadny pohyb bez podkladu</t>
+          <t>1,664 invoice payments (reference, company ID, amount) and 4,784 named internal payments — no movement without support</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>105 stredísk × mesiacov: mzdy == 521 a 524 (MD − D) na cent</t>
+          <t>105 cost centres × months: payroll == 521 and 524 (Dr − Cr) to the cent</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1,741 faktúr zaúčtovaných pod svojím číslom na správnom účte, stredisku, mesiaci a sume</t>
+          <t>1,741 invoices posted under their own number to the right account, cost centre, month and amount</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>84 stredísk × mesiacov: zásoby nezáporné a nadväzujú, stav == pohyby, príjem == 132, výdaj == 504</t>
+          <t>84 cost centres × months: stock non-negative and carried forward, levels == movements, received == 132, issued == 504</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31,758 riadkov denníka: každý na povolenej predkontácii (41 vzorov z profilu)</t>
+          <t>31,758 journal rows: each on an allowed posting pattern (41 patterns from the profile)</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>340 úhrad záväzkov (331, 336, 342, 341, 343) == záväzok predchádzajúceho mesiaca</t>
+          <t>340 liability payments (331, 336, 342, 341, 343) == liability of the previous month</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>84 predajní × mesiacov: poplatok 568 == tržby kartou − pripísané bankou; zostatok 315 == nepripísané tržby</t>
+          <t>84 stores × months: fee 568 == card sales − credited by the bank; balance 315 == sales not yet credited</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>21 mesiacov: úrok == zostatok × sadzba / 12 a splátka == zmluva</t>
+          <t>21 months: interest == balance × rate / 12 and repayment == agreement</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16 výnosových/nákladových účtov zaradených do výsledovky</t>
+          <t>16 income/expense accounts mapped to the P&amp;L</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>vykázané súčty == predvaha podľa účtovej politiky profilu na cent: Tržby, Hrubá marža, EBITDA, EBIT, Zisk pred zdanením, Čistý zisk (sumy sú v Prehľade, pri NESEDÍ sa nevydávajú)</t>
+          <t>reported totals == trial balance per the profile's accounting policy, to the cent: Revenue, Gross margin, EBITDA, EBIT, Profit before tax, Net profit (the amounts are in the Overview; on DOES NOT TIE they are not issued)</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>board pack == druhá cesta na cent: 660 buniek mriežky, 153 buniek odhadu, 96 riadkov (YTD, plán, minulý rok, odhad roka), odchýlky a poradie, 1 pravidiel rizík s €; plán úplný</t>
+          <t>board pack == second path to the cent: 660 grid cells, 153 forecast cells, 96 lines (YTD, plan, last year, full-year forecast), variances and their order, 1 risk rules with €; plan complete</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>108/108 čísel sedí s etalónom na cent</t>
+          <t>108/108 figures tie to the reference to the cent</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0 výnimiek v platnom tvare</t>
+          <t>0 exceptions in a valid form</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17/17 čísel zmluvy z hotového prehlad.xlsx sedí s 2 kotvami mimo motora (±1 €; percentá = správne zaokrúhlená kotva)</t>
+          <t>17/17 contract figures from the finished overview.xlsx tie to 2 anchors outside the engine (±€1; percentages = correctly rounded anchor)</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1334,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Kontrolný panel</t>
+          <t>Control panel</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -1354,12 +1354,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>stav k 2026-09</t>
+          <t>as of 2026-09</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Verdikt: SEDÍ</t>
+          <t>Verdict: TIES</t>
         </is>
       </c>
     </row>
@@ -1367,39 +1367,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Semafor</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Oblasť</t>
+          <t>Area</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kontrola</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Výsledok</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Nálezov</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Chybné riadky</t>
+          <t>Failed rows</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>dodávka = kontrakt (233 súborov)</t>
+          <t>delivery = contract (233 files)</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>382,560 riadkov z 10 tabuliek zdrojov prečítaných bez straty</t>
+          <t>382,560 rows from 10 source tables read without loss</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4,350 súm je číslo v dohodnutom tvare</t>
+          <t>4,350 amounts are numbers in the agreed format</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>bločky, denník, faktúry, mzdy, banka aj predvaha bez duplicít</t>
+          <t>receipts, journal, invoices, payroll, bank and trial balance without duplicates</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vstupy — tvar a úplnosť</t>
+          <t>Inputs — shape and completeness</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>21 mesiacov × 7 zdrojov a 4 pokladne × 21 mesiacov bez medzery</t>
+          <t>21 months × 7 sources and 4 POS × 21 months without a gap</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1531,7 +1531,7 @@
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>84 exportov pokladne: SPOLU == súčet bločkov</t>
+          <t>84 POS exports: TOTAL == sum of receipts</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2,175 obratov mesiac × stredisko × účet: denník == predvaha na cent</t>
+          <t>2,175 turnovers month × cost centre × account: journal == trial balance to the cent</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2,088 predajných dní × predajňa: bločky == 211/315 po spôsobe platby a tržby bez DPH == celý účet 604</t>
+          <t>2,088 sales days × store: receipts == 211/315 by payment method and revenue excl. VAT == the whole account 604</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>21 výpisov: zostatky nadväzujú a sedia s pohybmi</t>
+          <t>21 statements: balances carry forward and tie to the movements</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>439 bankových dní: výpis == účet 221 na cent</t>
+          <t>439 bank days: statement == account 221 to the cent</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1,664 úhrad faktúr (VS, IČO, suma) a 4,784 menovitých interných platieb — žiadny pohyb bez podkladu</t>
+          <t>1,664 invoice payments (reference, company ID, amount) and 4,784 named internal payments — no movement without support</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>105 stredísk × mesiacov: mzdy == 521 a 524 (MD − D) na cent</t>
+          <t>105 cost centres × months: payroll == 521 and 524 (Dr − Cr) to the cent</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,741 faktúr zaúčtovaných pod svojím číslom na správnom účte, stredisku, mesiaci a sume</t>
+          <t>1,741 invoices posted under their own number to the right account, cost centre, month and amount</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>84 stredísk × mesiacov: zásoby nezáporné a nadväzujú, stav == pohyby, príjem == 132, výdaj == 504</t>
+          <t>84 cost centres × months: stock non-negative and carried forward, levels == movements, received == 132, issued == 504</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>84 predajní × mesiacov: poplatok 568 == tržby kartou − pripísané bankou; zostatok 315 == nepripísané tržby</t>
+          <t>84 stores × months: fee 568 == card sales − credited by the bank; balance 315 == sales not yet credited</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>340 úhrad záväzkov (331, 336, 342, 341, 343) == záväzok predchádzajúceho mesiaca</t>
+          <t>340 liability payments (331, 336, 342, 341, 343) == liability of the previous month</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Párovania zdroj ↔ zdroj</t>
+          <t>Reconciliations source ↔ source</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>21 mesiacov: úrok == zostatok × sadzba / 12 a splátka == zmluva</t>
+          <t>21 months: interest == balance × rate / 12 and repayment == agreement</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1838,7 +1838,7 @@
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Účtovná logika a výsledovka</t>
+          <t>Accounting logic and P&amp;L</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Účtovná logika a výsledovka</t>
+          <t>Accounting logic and P&amp;L</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>31,758 riadkov denníka: každý na povolenej predkontácii (41 vzorov z profilu)</t>
+          <t>31,758 journal rows: each on an allowed posting pattern (41 patterns from the profile)</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Účtovná logika a výsledovka</t>
+          <t>Accounting logic and P&amp;L</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>16 výnosových/nákladových účtov zaradených do výsledovky</t>
+          <t>16 income/expense accounts mapped to the P&amp;L</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Účtovná logika a výsledovka</t>
+          <t>Accounting logic and P&amp;L</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>vykázané súčty == predvaha podľa účtovej politiky profilu na cent: Tržby, Hrubá marža, EBITDA, EBIT, Zisk pred zdanením, Čistý zisk (sumy sú v Prehľade, pri NESEDÍ sa nevydávajú)</t>
+          <t>reported totals == trial balance per the profile's accounting policy, to the cent: Revenue, Gross margin, EBITDA, EBIT, Profit before tax, Net profit (the amounts are in the Overview; on DOES NOT TIE they are not issued)</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Účtovná logika a výsledovka</t>
+          <t>Accounting logic and P&amp;L</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>board pack == druhá cesta na cent: 660 buniek mriežky, 153 buniek odhadu, 96 riadkov (YTD, plán, minulý rok, odhad roka), odchýlky a poradie, 1 pravidiel rizík s €; plán úplný</t>
+          <t>board pack == second path to the cent: 660 grid cells, 153 forecast cells, 96 lines (YTD, plan, last year, full-year forecast), variances and their order, 1 risk rules with €; plan complete</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1945,7 +1945,7 @@
     <row r="28">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Výstup a etalón</t>
+          <t>Output and reference</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Výstup a etalón</t>
+          <t>Output and reference</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>model 'retail_full', 21 kontrol profilu (povinné: 21/21)</t>
+          <t>model 'retail_full', 21 checks in the profile (required: 21/21)</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Výstup a etalón</t>
+          <t>Output and reference</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0 výnimiek v platnom tvare</t>
+          <t>0 exceptions in a valid form</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Výstup a etalón</t>
+          <t>Output and reference</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>108/108 čísel sedí s etalónom na cent</t>
+          <t>108/108 figures tie to the reference to the cent</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Výstup a etalón</t>
+          <t>Output and reference</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>17/17 čísel zmluvy z hotového prehlad.xlsx sedí s 2 kotvami mimo motora (±1 €; percentá = správne zaokrúhlená kotva)</t>
+          <t>17/17 contract figures from the finished overview.xlsx tie to 2 anchors outside the engine (±€1; percentages = correctly rounded anchor)</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2053,7 +2053,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Nad hotovým súborom bežia ešte xlsx_readback, control_panel_readback a pivot_pl_match — ich FAIL súbory zmaže; tento súbor existuje = prešli (výsledok na obrazovke behu a v logu).</t>
+          <t>On the finished file xlsx_readback, control_panel_readback and pivot_pl_match also run — their FAIL deletes the files; this file exists = they passed (result on the run screen and in the log).</t>
         </is>
       </c>
     </row>
@@ -2061,46 +2061,46 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Vstupy — čo prišlo</t>
+          <t>Inputs — what arrived</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Zdroj</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Súbory očakávané</t>
+          <t>Files expected</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Súbory prišli</t>
+          <t>Files received</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Riadky načítané</t>
+          <t>Rows read</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Nečitateľné riadky</t>
+          <t>Unreadable rows</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Semafor</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pokladňa — bločky</t>
+          <t>POS — receipts</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2124,7 +2124,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Účtovný denník</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2148,7 +2148,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Predvaha</t>
+          <t>Trial balance</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2172,7 +2172,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Faktúry dodávateľov</t>
+          <t>Supplier invoices</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2196,7 +2196,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mzdy</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2220,7 +2220,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Banka</t>
+          <t>Bank</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2244,7 +2244,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sklad — pohyby</t>
+          <t>Stock — movements</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -2268,7 +2268,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sklad — stavy</t>
+          <t>Stock — levels</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2292,7 +2292,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Plán</t>
+          <t>Plan</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -2316,7 +2316,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Číselníky</t>
+          <t>Master data</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2353,12 +2353,12 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2369,44 +2369,44 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Kontrola</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Súbory (miesto detekcie)</t>
+          <t>Files (where detected)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Riadok</t>
+          <t>Row</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Nález</t>
+          <t>Finding</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Otvoriť 1</t>
+          <t>Open 1</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Otvoriť 2</t>
+          <t>Open 2</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Otvoriť 3</t>
+          <t>Open 3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="E2" t="inlineStr">
         <is>
-          <t>žiadne nálezy — všetky kontroly prešli</t>
+          <t>no findings — all checks passed</t>
         </is>
       </c>
     </row>
@@ -2424,56 +2424,56 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Riadok</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Predajňa Centrum</t>
+          <t>Store Centrum</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko</t>
+          <t>Store Sídlisko</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Predajňa OC</t>
+          <t>Store OC</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Predajňa Mesto</t>
+          <t>Store Mesto</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Centrála</t>
+          <t>Head office</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Spolu</t>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tržby</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -2498,7 +2498,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Náklady na predaný tovar</t>
+          <t>Cost of goods sold</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -2523,7 +2523,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hrubá marža</t>
+          <t>Gross margin</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -2548,7 +2548,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Personál</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -2573,7 +2573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nájom</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -2598,7 +2598,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -2648,7 +2648,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Služby</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -2673,7 +2673,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ostatné</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -2723,7 +2723,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Odpisy</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -2773,7 +2773,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Úroky a finančné</t>
+          <t>Interest and financial</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
@@ -2798,7 +2798,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zisk pred zdanením</t>
+          <t>Profit before tax</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
@@ -2823,7 +2823,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Daň z príjmov</t>
+          <t>Income tax</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
@@ -2848,7 +2848,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Čistý zisk</t>
+          <t>Net profit</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
@@ -2885,48 +2885,48 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Mesiac</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Predajňa Centrum</t>
+          <t>Store Centrum</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko</t>
+          <t>Store Sídlisko</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Predajňa OC</t>
+          <t>Store OC</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Predajňa Mesto</t>
+          <t>Store Mesto</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Centrála</t>
+          <t>Head office</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Spolu</t>
+          <t>Total</t>
         </is>
       </c>
     </row>
@@ -3469,44 +3469,44 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Predajňa</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Plán YTD</t>
+          <t>Plan YTD</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Skutočnosť YTD</t>
+          <t>Actual YTD</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Rozdiel</t>
+          <t>Variance</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Plnenie</t>
+          <t>Achievement</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Predajňa Centrum</t>
+          <t>Store Centrum</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -3525,7 +3525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko</t>
+          <t>Store Sídlisko</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -3544,7 +3544,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Predajňa OC</t>
+          <t>Store OC</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -3563,7 +3563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Predajňa Mesto</t>
+          <t>Store Mesto</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -3582,7 +3582,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Centrála</t>
+          <t>Head office</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -3609,74 +3609,74 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Riadok</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>YTD skutočnosť</t>
+          <t>Actual YTD</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>YTD plán</t>
+          <t>Plan YTD</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Rozdiel voči plánu</t>
+          <t>Variance vs plan</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>YTD minulý rok</t>
+          <t>Last year YTD</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Rozdiel voči minulému roku</t>
+          <t>Variance vs last year</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Odhad roka</t>
+          <t>Full-year forecast</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Plán roka</t>
+          <t>Full-year plan</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Odhad − plán roka</t>
+          <t>Forecast − plan</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Minulý rok celý</t>
+          <t>Last year full</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tržby</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -3710,7 +3710,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Náklady na predaný tovar</t>
+          <t>Cost of goods sold</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -3744,7 +3744,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hrubá marža</t>
+          <t>Gross margin</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -3778,7 +3778,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Personál</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -3812,7 +3812,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nájom</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -3846,7 +3846,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -3914,7 +3914,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Služby</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -3948,7 +3948,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ostatné</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -4016,7 +4016,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Odpisy</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -4084,7 +4084,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Úroky a finančné</t>
+          <t>Interest and financial</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
@@ -4118,7 +4118,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zisk pred zdanením</t>
+          <t>Profit before tax</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
@@ -4152,7 +4152,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Daň z príjmov</t>
+          <t>Income tax</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
@@ -4186,7 +4186,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Čistý zisk</t>
+          <t>Net profit</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
@@ -4231,56 +4231,56 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Riadok</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Predajňa Centrum</t>
+          <t>Store Centrum</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko</t>
+          <t>Store Sídlisko</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Predajňa OC</t>
+          <t>Store OC</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Predajňa Mesto</t>
+          <t>Store Mesto</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Centrála</t>
+          <t>Head office</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Spolu</t>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tržby</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -4305,7 +4305,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Náklady na predaný tovar</t>
+          <t>Cost of goods sold</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -4330,7 +4330,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hrubá marža</t>
+          <t>Gross margin</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -4355,7 +4355,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Personál</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -4380,7 +4380,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nájom</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -4405,7 +4405,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -4455,7 +4455,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Služby</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -4480,7 +4480,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ostatné</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -4530,7 +4530,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Odpisy</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -4580,7 +4580,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Úroky a finančné</t>
+          <t>Interest and financial</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
@@ -4605,7 +4605,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zisk pred zdanením</t>
+          <t>Profit before tax</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
@@ -4630,7 +4630,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Daň z príjmov</t>
+          <t>Income tax</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
@@ -4655,7 +4655,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Čistý zisk</t>
+          <t>Net profit</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
@@ -4691,50 +4691,50 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="47" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Stredisko · riadok</t>
+          <t>Cost centre · line</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>YTD skutočnosť</t>
+          <t>Actual YTD</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>YTD plán</t>
+          <t>Plan YTD</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Vplyv na EBITDA voči plánu</t>
+          <t>EBITDA impact vs plan</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Vplyv voči minulému roku</t>
+          <t>Impact vs last year</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Príčina</t>
+          <t>Cause</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Predajňa OC · Nájom</t>
+          <t>Store OC · Rent</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -4751,14 +4751,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>od 2026-04 mesačne −2 600 €</t>
+          <t>since 2026-04, every month −€2,600</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Predajňa Mesto · Hrubá marža</t>
+          <t>Store Mesto · Gross margin</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -4775,14 +4775,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>najmä v Q2 (−2 692 €)</t>
+          <t>mainly in Q2 (−€2,692)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Predajňa OC · Hrubá marža</t>
+          <t>Store OC · Gross margin</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -4799,14 +4799,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>najmä v Q3 (+5 421 €)</t>
+          <t>mainly in Q3 (+€5,421)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko · Hrubá marža</t>
+          <t>Store Sídlisko · Gross margin</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>rozložené počas roka (priemer −365 € mesačne)</t>
+          <t>spread across the year (average −€365 per month)</t>
         </is>
       </c>
     </row>
@@ -4841,43 +4841,43 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="90" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Kľúč</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Typ</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Vplyv na EBITDA</t>
+          <t>EBITDA impact</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Popis</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ro|skok_nakladu|Energie|Q1</t>
+          <t>ro|cost_spike|Energy|Q1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>riziko</t>
+          <t>risk</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
@@ -4885,19 +4885,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Energie: v Q1 2026 +35,0 % medziročne, posledných 3 mesiacov +0,0 %; ak sa skok zopakuje vo zvyšku roka (minulý rok −5 083 € × 1,35), EBITDA −1 779 € voči odhadu.</t>
+          <t>Energy: in Q1 2026 +35.0% year on year, last 3 months +0.0%; if the spike repeats in the rest of the year (last year −€5,083 × 1.35), EBITDA −€1,779 vs forecast.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>citlivost|mix_kategorie|Papiernictvo</t>
+          <t>sensitivity|category_mix|Stationery</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>citlivosť odhadu</t>
+          <t>forecast sensitivity</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
@@ -4905,19 +4905,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Papiernictvo (rast +21,9 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 52,9 % tržieb, vo zvyšku roka 33,8 %; oprava na podiel zvyšku roka: EBITDA −9 783 € (× hrubá marža).</t>
+          <t>Stationery (growth +21.9% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 52.9% share of revenue, in the rest of the year 33.8%; correction to the rest-of-year share: EBITDA −€9,783 (× gross margin).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>citlivost|mix_kategorie|Hračky</t>
+          <t>sensitivity|category_mix|Toys</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>citlivosť odhadu</t>
+          <t>forecast sensitivity</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hračky (pokles −18,5 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 15,0 % tržieb, vo zvyšku roka 25,1 %; oprava na podiel zvyšku roka: EBITDA −4 356 € (× hrubá marža).</t>
+          <t>Toys (decline −18.5% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 15.0% share of revenue, in the rest of the year 25.1%; correction to the rest-of-year share: EBITDA −€4,356 (× gross margin).</t>
         </is>
       </c>
     </row>
@@ -4943,10 +4943,10 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4954,39 +4954,39 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Kľúč</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Číslo</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Komentár stroja</t>
+          <t>Machine comment</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Komentár kontrolóra</t>
+          <t>Controller comment</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Platný komentár</t>
+          <t>Valid comment</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Stav</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>odhad|Tržby</t>
+          <t>forecast|Revenue</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
@@ -4994,24 +4994,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tržby 2026 — odhad 2 122 954 €: voči plánu −8 532 € (−0,4 %), voči minulému roku +149 356 €; z toho skutočnosť 1 496 289 € a odhad zvyšku roka 626 665 €.</t>
+          <t>Revenue 2026 — forecast €2,122,954: vs plan −€8,532 (−0.4%), vs last year +€149,356; of which actual €1,496,289 and rest-of-year forecast €626,665.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tržby 2026 — odhad 2 122 954 €: voči plánu −8 532 € (−0,4 %), voči minulému roku +149 356 €; z toho skutočnosť 1 496 289 € a odhad zvyšku roka 626 665 €.</t>
+          <t>Revenue 2026 — forecast €2,122,954: vs plan −€8,532 (−0.4%), vs last year +€149,356; of which actual €1,496,289 and rest-of-year forecast €626,665.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>odhad|EBITDA</t>
+          <t>forecast|EBITDA</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -5019,24 +5019,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EBITDA 2026 — odhad 241 296 €: voči plánu −23 660 € (−8,9 %), voči minulému roku +19 825 €; z toho skutočnosť 160 045 € a odhad zvyšku roka 81 251 €.</t>
+          <t>EBITDA 2026 — forecast €241,296: vs plan −€23,660 (−8.9%), vs last year +€19,825; of which actual €160,045 and rest-of-year forecast €81,251.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EBITDA 2026 — odhad 241 296 €: voči plánu −23 660 € (−8,9 %), voči minulému roku +19 825 €; z toho skutočnosť 160 045 € a odhad zvyšku roka 81 251 €.</t>
+          <t>EBITDA 2026 — forecast €241,296: vs plan −€23,660 (−8.9%), vs last year +€19,825; of which actual €160,045 and rest-of-year forecast €81,251.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>odhad|Čistý zisk</t>
+          <t>forecast|Net profit</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
@@ -5044,24 +5044,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Čistý zisk 2026 — odhad 149 246 €: voči plánu −17 233 € (−10,4 %), voči minulému roku +17 120 €; z toho skutočnosť 95 279 € a odhad zvyšku roka 53 967 €.</t>
+          <t>Net profit 2026 — forecast €149,246: vs plan −€17,233 (−10.4%), vs last year +€17,120; of which actual €95,279 and rest-of-year forecast €53,967.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Čistý zisk 2026 — odhad 149 246 €: voči plánu −17 233 € (−10,4 %), voči minulému roku +17 120 €; z toho skutočnosť 95 279 € a odhad zvyšku roka 53 967 €.</t>
+          <t>Net profit 2026 — forecast €149,246: vs plan −€17,233 (−10.4%), vs last year +€17,120; of which actual €95,279 and rest-of-year forecast €53,967.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>odchylka|Predajňa OC|Nájom</t>
+          <t>variance|Store OC|Rent</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
@@ -5069,24 +5069,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Predajňa OC · Nájom: vplyv na EBITDA −15 600 € voči plánu (−31,0 %) — od 2026-04 mesačne −2 600 €; voči minulému roku −15 600 €.</t>
+          <t>Store OC · Rent: EBITDA impact −€15,600 vs plan (−31.0%) — since 2026-04, every month −€2,600; vs last year −€15,600.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Predajňa OC · Nájom: vplyv na EBITDA −15 600 € voči plánu (−31,0 %) — od 2026-04 mesačne −2 600 €; voči minulému roku −15 600 €.</t>
+          <t>Store OC · Rent: EBITDA impact −€15,600 vs plan (−31.0%) — since 2026-04, every month −€2,600; vs last year −€15,600.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>odchylka|Predajňa Mesto|Hrubá marža</t>
+          <t>variance|Store Mesto|Gross margin</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
@@ -5094,24 +5094,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Predajňa Mesto · Hrubá marža: vplyv na EBITDA −3 904 € voči plánu (−4,4 %) — najmä v Q2 (−2 692 €); voči minulému roku +2 735 €.</t>
+          <t>Store Mesto · Gross margin: EBITDA impact −€3,904 vs plan (−4.4%) — mainly in Q2 (−€2,692); vs last year +€2,735.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Predajňa Mesto · Hrubá marža: vplyv na EBITDA −3 904 € voči plánu (−4,4 %) — najmä v Q2 (−2 692 €); voči minulému roku +2 735 €.</t>
+          <t>Store Mesto · Gross margin: EBITDA impact −€3,904 vs plan (−4.4%) — mainly in Q2 (−€2,692); vs last year +€2,735.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>odchylka|Predajňa OC|Hrubá marža</t>
+          <t>variance|Store OC|Gross margin</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -5119,24 +5119,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Predajňa OC · Hrubá marža: vplyv na EBITDA +3 626 € voči plánu (+1,6 %) — najmä v Q3 (+5 421 €); voči minulému roku +20 919 €.</t>
+          <t>Store OC · Gross margin: EBITDA impact +€3,626 vs plan (+1.6%) — mainly in Q3 (+€5,421); vs last year +€20,919.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Predajňa OC · Hrubá marža: vplyv na EBITDA +3 626 € voči plánu (+1,6 %) — najmä v Q3 (+5 421 €); voči minulému roku +20 919 €.</t>
+          <t>Store OC · Gross margin: EBITDA impact +€3,626 vs plan (+1.6%) — mainly in Q3 (+€5,421); vs last year +€20,919.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>odchylka|Predajňa Sídlisko|Hrubá marža</t>
+          <t>variance|Store Sídlisko|Gross margin</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
@@ -5144,24 +5144,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko · Hrubá marža: vplyv na EBITDA −3 286 € voči plánu (−2,7 %) — rozložené počas roka (priemer −365 € mesačne); voči minulému roku +5 738 €.</t>
+          <t>Store Sídlisko · Gross margin: EBITDA impact −€3,286 vs plan (−2.7%) — spread across the year (average −€365 per month); vs last year +€5,738.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Predajňa Sídlisko · Hrubá marža: vplyv na EBITDA −3 286 € voči plánu (−2,7 %) — rozložené počas roka (priemer −365 € mesačne); voči minulému roku +5 738 €.</t>
+          <t>Store Sídlisko · Gross margin: EBITDA impact −€3,286 vs plan (−2.7%) — spread across the year (average −€365 per month); vs last year +€5,738.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ro|skok_nakladu|Energie|Q1</t>
+          <t>ro|cost_spike|Energy|Q1</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
@@ -5169,24 +5169,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Energie: v Q1 2026 +35,0 % medziročne, posledných 3 mesiacov +0,0 %; ak sa skok zopakuje vo zvyšku roka (minulý rok −5 083 € × 1,35), EBITDA −1 779 € voči odhadu.</t>
+          <t>Energy: in Q1 2026 +35.0% year on year, last 3 months +0.0%; if the spike repeats in the rest of the year (last year −€5,083 × 1.35), EBITDA −€1,779 vs forecast.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Energie: v Q1 2026 +35,0 % medziročne, posledných 3 mesiacov +0,0 %; ak sa skok zopakuje vo zvyšku roka (minulý rok −5 083 € × 1,35), EBITDA −1 779 € voči odhadu.</t>
+          <t>Energy: in Q1 2026 +35.0% year on year, last 3 months +0.0%; if the spike repeats in the rest of the year (last year −€5,083 × 1.35), EBITDA −€1,779 vs forecast.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>citlivost|mix_kategorie|Papiernictvo</t>
+          <t>sensitivity|category_mix|Stationery</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -5194,24 +5194,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Papiernictvo (rast +21,9 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 52,9 % tržieb, vo zvyšku roka 33,8 %; oprava na podiel zvyšku roka: EBITDA −9 783 € (× hrubá marža).</t>
+          <t>Stationery (growth +21.9% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 52.9% share of revenue, in the rest of the year 33.8%; correction to the rest-of-year share: EBITDA −€9,783 (× gross margin).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Papiernictvo (rast +21,9 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 52,9 % tržieb, vo zvyšku roka 33,8 %; oprava na podiel zvyšku roka: EBITDA −9 783 € (× hrubá marža).</t>
+          <t>Stationery (growth +21.9% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 52.9% share of revenue, in the rest of the year 33.8%; correction to the rest-of-year share: EBITDA −€9,783 (× gross margin).</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>citlivost|mix_kategorie|Hračky</t>
+          <t>sensitivity|category_mix|Toys</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
@@ -5219,24 +5219,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hračky (pokles −18,5 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 15,0 % tržieb, vo zvyšku roka 25,1 %; oprava na podiel zvyšku roka: EBITDA −4 356 € (× hrubá marža).</t>
+          <t>Toys (decline −18.5% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 15.0% share of revenue, in the rest of the year 25.1%; correction to the rest-of-year share: EBITDA −€4,356 (× gross margin).</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hračky (pokles −18,5 % medziročne v Q3, 3. štvrťrok po sebe): ak medziročný trend pokračuje, tempo posledných 3 mesiacov nadhodnocuje odhad — v rovnakých mesiacoch minulého roka mala kategória podiel 15,0 % tržieb, vo zvyšku roka 25,1 %; oprava na podiel zvyšku roka: EBITDA −4 356 € (× hrubá marža).</t>
+          <t>Toys (decline −18.5% year on year in Q3, 3 quarters in a row): if the year-on-year trend continues, the pace of the last 3 months overstates the forecast — in the same months of last year the category had a 15.0% share of revenue, in the rest of the year 25.1%; correction to the rest-of-year share: EBITDA −€4,356 (× gross margin).</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>board|category_decline|Hračky</t>
+          <t>board|category_decline|Toys</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -5244,17 +5244,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hračky: medziročný pokles 3 štvrťroky po sebe (Q1 −6,8 %, Q2 −13,5 %, Q3 −18,5 %)</t>
+          <t>Toys: year-on-year decline 3 quarters in a row (Q1 −6.8%, Q2 −13.5%, Q3 −18.5%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hračky: medziročný pokles 3 štvrťroky po sebe (Q1 −6,8 %, Q2 −13,5 %, Q3 −18,5 %)</t>
+          <t>Toys: year-on-year decline 3 quarters in a row (Q1 −6.8%, Q2 −13.5%, Q3 −18.5%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>stroj</t>
+          <t>machine</t>
         </is>
       </c>
     </row>

</xml_diff>